<commit_message>
Move the Sprint 1 close standup from Friday 23 October to Thursday 22.
Friday 23 stays a zero-hour buffer day with no Daily Scrum.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/sprint-1-backlog-conclusion.xlsx
+++ b/docs/sprint-1-backlog-conclusion.xlsx
@@ -2201,7 +2201,7 @@
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="12" t="inlineStr">
         <is>
-          <t>Sprint 1 conclusion. Same W02 columns as the planning sheet (ID, User Story, Tasks, Owner, Status, Estimated effort, Day 1–15). Day cells are actual hours logged and match the Daily Scrum scripts: Meeting 3 = Day 2 (8h); Meeting 4 = Days 3–4 (22h); Meeting 5 = Days 5–8 (41h); Meeting 6 = Days 9–14 (39h); Day 1 (4h) is Meeting 2; Day 15 buffer is 0. Status is Done after Meeting 6 DoD. Remaining effort is 0. See sheet Standup map. This Done column is the Friday 23 October result after Meeting 6. On Friday 16 October (Meeting 3) the live board is Day 2 only. Sprint 2 stories (US3b, US4a, US4b, US5b, US7, US8) stay on the product backlog.</t>
+          <t>Sprint 1 conclusion. Same W02 columns as the planning sheet (ID, User Story, Tasks, Owner, Status, Estimated effort, Day 1–15). Day cells are actual hours logged and match the Daily Scrum scripts: Meeting 3 = Day 2 (8h); Meeting 4 = Days 3–4 (22h); Meeting 5 = Days 5–8 (41h); Meeting 6 = Days 9–14 (39h); Day 1 (4h) is Meeting 2; Day 15 buffer is 0. Status is Done after Meeting 6 DoD. Remaining effort is 0. See sheet Standup map. This Done column is the Thursday 22 October result after Meeting 6. On Friday 16 October (Meeting 3) the live board is Day 2 only. Sprint 2 stories (US3b, US4a, US4b, US5b, US7, US8) stay on the product backlog.</t>
         </is>
       </c>
     </row>
@@ -2448,7 +2448,7 @@
       </c>
       <c r="B9" s="16" t="inlineStr">
         <is>
-          <t>Fri 23 Oct 2026</t>
+          <t>Thu 22 Oct 2026</t>
         </is>
       </c>
       <c r="C9" s="17" t="inlineStr">
@@ -2642,7 +2642,7 @@
     <row r="20">
       <c r="A20" s="12" t="inlineStr">
         <is>
-          <t>Today is Friday 16 October (Meeting 3): live board is Day 2 only. Meeting 4 must not say US6 is built (Days 6-8, Meeting 5). Meeting 5 must not say US2a incoming or US2b are finished (Days 9-11, Meeting 6). US1a moves to Done at Meeting 5. Remaining 0 only after Meeting 6 on Friday 23 October. Sprint 2 (US3b, US4a, US4b, US5b, US7, US8) is not Sprint 1 Done.</t>
+          <t>Today is Friday 16 October (Meeting 3): live board is Day 2 only. Meeting 4 must not say US6 is built (Days 6-8, Meeting 5). Meeting 5 must not say US2a incoming or US2b are finished (Days 9-11, Meeting 6). US1a moves to Done at Meeting 5. Remaining 0 only after Meeting 6 on Thursday 22 October. Friday 23 has no standup. Sprint 2 (US3b, US4a, US4b, US5b, US7, US8) is not Sprint 1 Done.</t>
         </is>
       </c>
     </row>

</xml_diff>